<commit_message>
Versão inicial do Dashboard Master Prime
</commit_message>
<xml_diff>
--- a/vagas_veiculos_pesados.xlsx
+++ b/vagas_veiculos_pesados.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>VP039</t>
+          <t>VP040</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>R$ 2.305,88</t>
+          <t>R$ 2.554,60</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>111 meses</t>
+          <t>110 meses</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>66,90%</t>
+          <t>68,02%</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>569/600</t>
+          <t>598/600</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>VP036</t>
+          <t>VP039</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>R$ 2.380,72</t>
+          <t>R$ 2.554,60</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -578,17 +578,17 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>110 meses</t>
+          <t>109 meses</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>64,58%</t>
+          <t>69,30%</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>546/600</t>
+          <t>597/600</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -600,7 +600,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>VP035</t>
+          <t>VP038</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>R$ 2.305,88</t>
+          <t>R$ 2.554,60</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -625,17 +625,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>108 meses</t>
+          <t>110 meses</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>63,36%</t>
+          <t>69,79%</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>599/600</t>
+          <t>597/600</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>VP034</t>
+          <t>VP036</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>R$ 2.162,60</t>
+          <t>R$ 2.380,72</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -672,17 +672,17 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>106 meses</t>
+          <t>108 meses</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>65,49%</t>
+          <t>65,09%</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>526/600</t>
+          <t>582/600</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -694,7 +694,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>VP031</t>
+          <t>VP034</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>R$ 2.293,69</t>
+          <t>R$ 2.162,60</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -719,17 +719,17 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>102 meses</t>
+          <t>104 meses</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>63,89%</t>
+          <t>62,26%</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>559/600</t>
+          <t>597/600</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>VP030</t>
+          <t>VP033</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -766,17 +766,17 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>101 meses</t>
+          <t>100 meses</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>64,30%</t>
+          <t>60,03%</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>545/600</t>
+          <t>599/600</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -788,7 +788,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>VP029</t>
+          <t>VP031</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -813,17 +813,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>101 meses</t>
+          <t>100 meses</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>62,96%</t>
+          <t>63,96%</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>595/600</t>
+          <t>597/600</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -835,7 +835,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>VP028</t>
+          <t>VP030</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -860,17 +860,17 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>100 meses</t>
+          <t>99 meses</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>64,25%</t>
+          <t>63,71%</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>539/600</t>
+          <t>594/600</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -882,7 +882,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>VP027</t>
+          <t>VP028</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -907,17 +907,17 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>97 meses</t>
+          <t>98 meses</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>60,20%</t>
+          <t>62,37%</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>574/600</t>
+          <t>537/600</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -929,7 +929,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>VP026</t>
+          <t>VP027</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -954,17 +954,17 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>96 meses</t>
+          <t>95 meses</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>62,86%</t>
+          <t>63,48%</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>536/600</t>
+          <t>562/600</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -976,7 +976,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>VP025</t>
+          <t>VP026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>R$ 1.945,93</t>
+          <t>R$ 2.293,69</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1001,17 +1001,17 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>93 meses</t>
+          <t>94 meses</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>59,19%</t>
+          <t>60,93%</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>564/600</t>
+          <t>531/600</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>VP024</t>
+          <t>VP025</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>R$ 2.293,69</t>
+          <t>R$ 1.945,93</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1048,17 +1048,17 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>90 meses</t>
+          <t>91 meses</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>59,58%</t>
+          <t>58,14%</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>591/600</t>
+          <t>567/600</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1070,7 +1070,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>VP023</t>
+          <t>VP024</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1100,12 +1100,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>57,03%</t>
+          <t>58,68%</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>590/600</t>
+          <t>589/600</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1117,7 +1117,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>VP022</t>
+          <t>VP023</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>88 meses</t>
+          <t>86 meses</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>61,12%</t>
+          <t>55,87%</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>578/600</t>
+          <t>598/600</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1164,7 +1164,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>VP021</t>
+          <t>VP022</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1189,17 +1189,17 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>88 meses</t>
+          <t>86 meses</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>60,76%</t>
+          <t>58,95%</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>594/600</t>
+          <t>572/600</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>VP020</t>
+          <t>VP021</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>R$ 1.941,89</t>
+          <t>R$ 2.293,69</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1241,12 +1241,12 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>57,21%</t>
+          <t>57,64%</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>337/360</t>
+          <t>593/600</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1258,12 +1258,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>VP019</t>
+          <t>VP020</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>R$ 190.000,00</t>
+          <t>R$ 180.000,00</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>R$ 1.968,21</t>
+          <t>R$ 2.202,35</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1283,17 +1283,17 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>85 meses</t>
+          <t>84 meses</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>57,35%</t>
+          <t>59,50%</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>347/360</t>
+          <t>338/360</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1305,12 +1305,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>VP018</t>
+          <t>VP019</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>R$ 180.000,00</t>
+          <t>R$ 190.000,00</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>R$ 1.941,89</t>
+          <t>R$ 1.968,21</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>65,77%</t>
+          <t>57,61%</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>356/360</t>
+          <t>355/360</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>VP017</t>
+          <t>VP018</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1377,17 +1377,17 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>79 meses</t>
+          <t>81 meses</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>55,88%</t>
+          <t>62,81%</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>359/360</t>
+          <t>350/360</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1424,67 +1424,20 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>76 meses</t>
+          <t>74 meses</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>60,14%</t>
+          <t>59,30%</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>353/360</t>
+          <t>357/360</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Ver grupo</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>VP012</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>R$ 200.000,00</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>R$ 360.000,00</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.187,42</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>120 meses</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>67 meses</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>59,48%</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>359/360</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Ver grupo</t>
         </is>
@@ -1512,7 +1465,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>16/04/2026 as 14:43:37</t>
+          <t>26/05/2026 as 10:18:24</t>
         </is>
       </c>
     </row>

</xml_diff>